<commit_message>
docs: Update test cases evidence to 15 cases with signature
</commit_message>
<xml_diff>
--- a/Evidencia_GA9-220501096-AA2-EV01_CasosPrueba.xlsx
+++ b/Evidencia_GA9-220501096-AA2-EV01_CasosPrueba.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Prueba" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de Prueba (15)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,13 +29,13 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -46,7 +46,7 @@
     <font>
       <name val="Calibri"/>
       <color rgb="00202020"/>
-      <sz val="10"/>
+      <sz val="9.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -540,26 +540,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SERVICIO NACIONAL DE APRENDIZAJE - SENA</t>
+          <t>SERVICIO NACIONAL DE APRENDIZAJE - SENA | REGIONAL ANTIOQUIA</t>
         </is>
       </c>
     </row>
@@ -645,12 +645,12 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Fecha de Ejecución:</t>
+          <t>Total de Casos:</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Septiembre 2026</t>
+          <t>15 Casos Diseñados y Aprobados</t>
         </is>
       </c>
       <c r="I6" s="5" t="n"/>
@@ -660,7 +660,7 @@
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1. DEFINICIÓN DEL AMBIENTE DE PRUEBAS</t>
+          <t>1. DEFINICIÓN DEL AMBIENTE DE PRUEBAS DE SOFTWARE</t>
         </is>
       </c>
     </row>
@@ -709,14 +709,14 @@
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Servidor de Backend</t>
+          <t>Servidor Backend</t>
         </is>
       </c>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Node.js v18+ con Framework Express.js en puerto local http://localhost:4000</t>
+          <t>Node.js v18+ con Express.js escuchando en http://localhost:4000</t>
         </is>
       </c>
       <c r="E11" s="5" t="n"/>
@@ -730,14 +730,14 @@
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Motor de Base de Datos</t>
+          <t>Base de Datos</t>
         </is>
       </c>
       <c r="B12" s="5" t="n"/>
       <c r="C12" s="5" t="n"/>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>MySQL Server 8.0 en puerto 3306 (Base de datos: camila_nails)</t>
+          <t>MySQL Server 8.0 en puerto 3306 (Base: camila_nails con motor InnoDB)</t>
         </is>
       </c>
       <c r="E12" s="5" t="n"/>
@@ -751,14 +751,14 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Frontend / Cliente Web</t>
+          <t>Cliente Frontend</t>
         </is>
       </c>
       <c r="B13" s="5" t="n"/>
       <c r="C13" s="5" t="n"/>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>React.js empaquetado con Vite en entorno http://localhost:5173</t>
+          <t>React.js empaquetado con Vite ejecutándose en http://localhost:5173</t>
         </is>
       </c>
       <c r="E13" s="5" t="n"/>
@@ -772,14 +772,14 @@
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Navegadores de Prueba</t>
+          <t>Navegadores</t>
         </is>
       </c>
       <c r="B14" s="5" t="n"/>
       <c r="C14" s="5" t="n"/>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Google Chrome v128+ y Microsoft Edge para pruebas de compatibilidad y DevTools</t>
+          <t>Google Chrome v128+ y Microsoft Edge (Pruebas de visualización y responsividad)</t>
         </is>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -793,14 +793,14 @@
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Herramientas de Pruebas</t>
+          <t>Herramientas de Prueba</t>
         </is>
       </c>
       <c r="B15" s="5" t="n"/>
       <c r="C15" s="5" t="n"/>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Postman v10+ (Pruebas de API REST / Endpoints) y Chrome DevTools (Pruebas de UI/Responsivo)</t>
+          <t>Postman v10+ (Pruebas de API REST) y Chrome DevTools (Inspección UI / CSS)</t>
         </is>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -814,7 +814,7 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>2. FORMATO DE MATRIZ DE CASOS DE PRUEBA</t>
+          <t>2. MATRIZ DE CASOS DE PRUEBA (15 CASOS DETALLADOS SEGÚN PROYECTO)</t>
         </is>
       </c>
     </row>
@@ -893,7 +893,7 @@
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
-          <t>Registro exitoso de nuevo usuario cliente (POST /api/register)</t>
+          <t>Registro exitoso de nuevo cliente (POST /api/register)</t>
         </is>
       </c>
       <c r="E19" s="13" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>Respuesta JSON status 200 en Postman y registro en base de datos</t>
+          <t>Respuesta JSON status 200 en Postman y persistencia en DB</t>
         </is>
       </c>
       <c r="K19" s="15" t="inlineStr">
@@ -955,12 +955,12 @@
       </c>
       <c r="E20" s="18" t="inlineStr">
         <is>
-          <t>Código HTTP 400 Bad Request con mensaje de error {'error': 'Faltan campos'}</t>
+          <t>Código HTTP 400 Bad Request con mensaje {'error': 'Faltan campos'}</t>
         </is>
       </c>
       <c r="F20" s="18" t="inlineStr">
         <is>
-          <t>Código HTTP 400 Bad Request retornado correctamente evitando registros incompletos</t>
+          <t>Código HTTP 400 Bad Request devuelto, bloqueando inserción incompleta</t>
         </is>
       </c>
       <c r="G20" s="14" t="inlineStr">
@@ -980,7 +980,7 @@
       </c>
       <c r="J20" s="18" t="inlineStr">
         <is>
-          <t>Captura de pantalla de Postman con código 400 y mensaje de validación</t>
+          <t>Captura de pantalla en Postman con respuesta 400 Bad Request</t>
         </is>
       </c>
       <c r="K20" s="15" t="inlineStr">
@@ -1007,17 +1007,17 @@
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Autenticación de usuario administrador en sistema (POST /api/login)</t>
+          <t>Control de usuario duplicado en registro (POST /api/register con email existente)</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Código HTTP 200 OK retornando datos de usuario y validación de rol 'admin'</t>
+          <t>Código HTTP 409 Conflict con mensaje {'error': 'Usuario o email ya existe'}</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>Acceso otorgado correctamente con datos de perfil y rol de administrador</t>
+          <t>Código HTTP 409 Conflict recibido impidiendo duplicidad de cuentas</t>
         </is>
       </c>
       <c r="G21" s="14" t="inlineStr">
@@ -1032,12 +1032,12 @@
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Media</t>
         </is>
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>Validación de contraseña encriptada con bcryptjs y sesión iniciada</t>
+          <t>Validación de restricción UNIQUE en MySQL retornando 409 en Postman</t>
         </is>
       </c>
       <c r="K21" s="15" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="B22" s="16" t="inlineStr">
         <is>
-          <t>Postman / Chrome</t>
+          <t>Postman</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
@@ -1064,17 +1064,17 @@
       </c>
       <c r="D22" s="18" t="inlineStr">
         <is>
-          <t>Creación manual de Ficha de Cliente desde Panel de Admin (POST /api/fichas)</t>
+          <t>Autenticación exitosa de usuario administrador (POST /api/login)</t>
         </is>
       </c>
       <c r="E22" s="18" t="inlineStr">
         <is>
-          <t>Registro insertado en tabla 'fichas' con ID autoincremental y mensaje de éxito</t>
+          <t>Código HTTP 200 OK con datos de perfil y validación de rol 'admin'</t>
         </is>
       </c>
       <c r="F22" s="18" t="inlineStr">
         <is>
-          <t>Ficha creada satisfactoriamente con Status 200 OK e insertId asignado</t>
+          <t>Acceso otorgado con status 200 OK y confirmación de rol administrativo</t>
         </is>
       </c>
       <c r="G22" s="14" t="inlineStr">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="J22" s="18" t="inlineStr">
         <is>
-          <t>Inserción reflejada en MySQL y visualización en tiempo real en la UI</t>
+          <t>Contraseña validada con hash bcryptjs y retorno de sesión en Postman</t>
         </is>
       </c>
       <c r="K22" s="15" t="inlineStr">
@@ -1121,17 +1121,17 @@
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Actualización y edición de datos de cliente (PUT /api/fichas/:id)</t>
+          <t>Rechazo de inicio de sesión con contraseña errada (POST /api/login)</t>
         </is>
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Modificación exitosa de nombre, teléfono y servicio devolviendo confirmación</t>
+          <t>Código HTTP 401 Unauthorized con mensaje {'error': 'Contraseña incorrecta'}</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Campos modificados en base de datos con respuesta {'message': 'Ficha actualizada'}</t>
+          <t>Código HTTP 401 recibido, impidiendo accesos no autorizados al sistema</t>
         </is>
       </c>
       <c r="G23" s="14" t="inlineStr">
@@ -1146,12 +1146,12 @@
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
-          <t>Petición PUT 200 OK en Postman y actualización visual en la tabla</t>
+          <t>Respuesta HTTP 401 Unauthorized documentada en Postman</t>
         </is>
       </c>
       <c r="K23" s="15" t="inlineStr">
@@ -1178,17 +1178,17 @@
       </c>
       <c r="D24" s="18" t="inlineStr">
         <is>
-          <t>Eliminación física de un usuario o ficha (DELETE /api/users/:id)</t>
+          <t>Consulta general de usuarios registrados (GET /api/users)</t>
         </is>
       </c>
       <c r="E24" s="18" t="inlineStr">
         <is>
-          <t>Registro eliminado de la base de datos MySQL con status 200 OK</t>
+          <t>Arreglo JSON con usuarios y campos públicos excluyendo contraseñas</t>
         </is>
       </c>
       <c r="F24" s="18" t="inlineStr">
         <is>
-          <t>Status 200 OK {'message': 'Usuario eliminado'} y registro borrado en DB</t>
+          <t>Respuesta 200 OK con lista completa de usuarios protegida sin hash</t>
         </is>
       </c>
       <c r="G24" s="14" t="inlineStr">
@@ -1203,12 +1203,12 @@
       </c>
       <c r="I24" s="16" t="inlineStr">
         <is>
-          <t>Media</t>
+          <t>Baja</t>
         </is>
       </c>
       <c r="J24" s="18" t="inlineStr">
         <is>
-          <t>Comprobación de registro ausente tras petición DELETE ejecutada</t>
+          <t>Array de usuarios en formato JSON retornado con Status 200 OK</t>
         </is>
       </c>
       <c r="K24" s="15" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="B25" s="11" t="inlineStr">
         <is>
-          <t>Chrome DevTools</t>
+          <t>Postman</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
@@ -1235,17 +1235,17 @@
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>Contraste y visibilidad de inputs en Modo Oscuro (Formularios Admin)</t>
+          <t>Modificación de rol de usuario (PATCH /api/users/:id/role)</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>El texto debe ser claramente legible (blanco sobre fondo oscuro) al escribir</t>
+          <t>Cambio de rol de 'user' a 'admin' reflejado en base de datos con status 200 OK</t>
         </is>
       </c>
       <c r="F25" s="13" t="inlineStr">
         <is>
-          <t>Se detectó fondo blanco en focus que ocultaba texto blanco; corregido en CSS</t>
+          <t>Rol actualizado exitosamente y verificado con consulta posterior</t>
         </is>
       </c>
       <c r="G25" s="14" t="inlineStr">
@@ -1255,7 +1255,7 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>BUG-UI-01</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
@@ -1265,7 +1265,7 @@
       </c>
       <c r="J25" s="13" t="inlineStr">
         <is>
-          <t>Regla CSS modificada (App.css) e inspección exitosa en DevTools</t>
+          <t>Respuesta PATCH status 200 OK con confirmación de cambio de rol</t>
         </is>
       </c>
       <c r="K25" s="15" t="inlineStr">
@@ -1282,50 +1282,449 @@
       </c>
       <c r="B26" s="16" t="inlineStr">
         <is>
+          <t>Postman / Chrome</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>Edición de datos de usuario en panel admin (PUT /api/users/:id)</t>
+        </is>
+      </c>
+      <c r="E26" s="18" t="inlineStr">
+        <is>
+          <t>Actualización de nombre y correo electrónico con confirmación 200 OK</t>
+        </is>
+      </c>
+      <c r="F26" s="18" t="inlineStr">
+        <is>
+          <t>Datos actualizados en MySQL y reflejados en el formulario en vivo</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H26" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="J26" s="18" t="inlineStr">
+        <is>
+          <t>Respuesta PUT 200 OK {'message': 'Usuario actualizado'}</t>
+        </is>
+      </c>
+      <c r="K26" s="15" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>CP-009</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Postman / Chrome</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
+        <is>
+          <t>Eliminación física de usuario desde panel (DELETE /api/users/:id)</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="inlineStr">
+        <is>
+          <t>Eliminación del registro con confirmación previa y respuesta 200 OK</t>
+        </is>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK {'message': 'Usuario eliminado'} y registro removido</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I27" s="11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J27" s="13" t="inlineStr">
+        <is>
+          <t>Comprobación de registro ausente tras petición DELETE ejecutada</t>
+        </is>
+      </c>
+      <c r="K27" s="15" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
+          <t>CP-010</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>Postman / Chrome</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+      <c r="D28" s="18" t="inlineStr">
+        <is>
+          <t>Creación manual de Ficha de Cliente desde Panel (POST /api/fichas)</t>
+        </is>
+      </c>
+      <c r="E28" s="18" t="inlineStr">
+        <is>
+          <t>Inserción en tabla 'fichas' con ID autoincremental y status 200 OK</t>
+        </is>
+      </c>
+      <c r="F28" s="18" t="inlineStr">
+        <is>
+          <t>Ficha creada con éxito, status 200 OK y asignación de insertId</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H28" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="J28" s="18" t="inlineStr">
+        <is>
+          <t>Ficha persistida en MySQL y visible de inmediato en la lista del panel</t>
+        </is>
+      </c>
+      <c r="K28" s="15" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t>CP-011</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Postman</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
+        <is>
+          <t>Consulta y listado histórico de Fichas Clínicas (GET /api/fichas)</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Retorno de todas las fichas ordenadas cronológicamente con status 200</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
+        <is>
+          <t>Arreglo JSON recibido con todos los historiales y servicios registrados</t>
+        </is>
+      </c>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="inlineStr">
+        <is>
+          <t>Baja</t>
+        </is>
+      </c>
+      <c r="J29" s="13" t="inlineStr">
+        <is>
+          <t>Respuesta GET 200 OK visualizada en Postman con arreglo de fichas</t>
+        </is>
+      </c>
+      <c r="K29" s="15" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>CP-012</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>Postman / Chrome</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>Actualización y edición de Ficha de Cliente (PUT /api/fichas/:id)</t>
+        </is>
+      </c>
+      <c r="E30" s="18" t="inlineStr">
+        <is>
+          <t>Modificación de teléfono y servicio asignado con status 200 OK</t>
+        </is>
+      </c>
+      <c r="F30" s="18" t="inlineStr">
+        <is>
+          <t>Campos modificados en MySQL con mensaje {'message': 'Ficha actualizada'}</t>
+        </is>
+      </c>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H30" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="J30" s="18" t="inlineStr">
+        <is>
+          <t>Petición PUT 200 OK en Postman y sincronización en interfaz React</t>
+        </is>
+      </c>
+      <c r="K30" s="15" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>CP-013</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Postman / Chrome</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Eliminación física de Ficha de Cliente (DELETE /api/fichas/:id)</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Registro de ficha eliminado de la base de datos con status 200 OK</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr">
+        <is>
+          <t>Status 200 OK {'message': 'Ficha eliminada'} y registro borrado en DB</t>
+        </is>
+      </c>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="J31" s="13" t="inlineStr">
+        <is>
+          <t>Comprobación en tabla 'fichas' y actualización de la lista en React</t>
+        </is>
+      </c>
+      <c r="K31" s="15" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="42" customHeight="1">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>CP-014</t>
+        </is>
+      </c>
+      <c r="B32" s="16" t="inlineStr">
+        <is>
           <t>Chrome DevTools</t>
         </is>
       </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>Andrés Mauricio Valencia Arango</t>
-        </is>
-      </c>
-      <c r="D26" s="18" t="inlineStr">
-        <is>
-          <t>Diseño responsivo del Home y Panel en dispositivos móviles (360px a 412px)</t>
-        </is>
-      </c>
-      <c r="E26" s="18" t="inlineStr">
-        <is>
-          <t>Adaptación fluida de columnas a 1 sola columna sin scroll horizontal indeseado</t>
-        </is>
-      </c>
-      <c r="F26" s="18" t="inlineStr">
-        <is>
-          <t>Reorganización de layout exitosa con padding adecuado para móviles y tablets</t>
-        </is>
-      </c>
-      <c r="G26" s="14" t="inlineStr">
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+      <c r="D32" s="18" t="inlineStr">
+        <is>
+          <t>Contraste y legibilidad de inputs en Modo Oscuro (Formularios Admin)</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>El texto debe ser claramente legible (blanco sobre fondo oscuro) al escribir</t>
+        </is>
+      </c>
+      <c r="F32" s="18" t="inlineStr">
+        <is>
+          <t>Se detectó fondo blanco en focus que ocultaba la letra; fue corregido en App.css</t>
+        </is>
+      </c>
+      <c r="G32" s="14" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="H26" s="16" t="inlineStr">
+      <c r="H32" s="16" t="inlineStr">
+        <is>
+          <t>BUG-UI-01</t>
+        </is>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="J32" s="18" t="inlineStr">
+        <is>
+          <t>Regla CSS modificada (App.css) e inspección exitosa en DevTools</t>
+        </is>
+      </c>
+      <c r="K32" s="15" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>CP-015</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Chrome DevTools</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Valencia Arango</t>
+        </is>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Diseño responsivo del Home y Navbar en móviles (360px a 412px)</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>Adaptación fluida de lado a lado sin marco rígido ni desbordamiento lateral</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Ancho fijo de 1126px reemplazado por 100% fluido con padding móvil perfecto</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="I26" s="16" t="inlineStr">
+      <c r="I33" s="11" t="inlineStr">
         <is>
           <t>Baja</t>
         </is>
       </c>
-      <c r="J26" s="18" t="inlineStr">
-        <is>
-          <t>Inspección en modo emulación responsive de Google Chrome</t>
-        </is>
-      </c>
-      <c r="K26" s="15" t="inlineStr">
+      <c r="J33" s="13" t="inlineStr">
+        <is>
+          <t>Emulación responsive en Google Chrome DevTools con visual amplia</t>
+        </is>
+      </c>
+      <c r="K33" s="15" t="inlineStr">
         <is>
           <t>Andrés Mauricio Valencia Arango</t>
         </is>

</xml_diff>